<commit_message>
actualizacion calendario html css js
</commit_message>
<xml_diff>
--- a/data/fokito/misiones.xlsx
+++ b/data/fokito/misiones.xlsx
@@ -12,9 +12,9 @@
     <sheet name="Plan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Misiones'!$A$1:$H$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matriz'!$A$1:$E$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Plan'!$A$1:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Misiones'!$A$1:$H$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Matriz'!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Plan'!$A$1:$H$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,16 +468,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="51" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -525,24 +525,24 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46134</v>
+        <v>46150</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46148</v>
+        <v>46136</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Trabajo práctico</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>pedir_preguntas</t>
+          <t>revisar_tp</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Cada profesor: 2 alternativas + 1 desarrollo (según tema de la prueba).</t>
+          <t>Revisar TP y poner nota. — Entrega al final</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -563,34 +563,34 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46141</v>
+        <v>46195</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46148</v>
+        <v>46216</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>construir_control</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>p6, p1</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Armar versión final, diagramación y revisión cruzada.</t>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -601,34 +601,34 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>46143</v>
+        <v>46195</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>46148</v>
+        <v>46216</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>pauta_prueba</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>p2, p5</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pauta oficial: dividir en 2 mitades si son 2 responsables.</t>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -639,34 +639,34 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>46145</v>
+        <v>46197</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>46148</v>
+        <v>46218</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>revisar_prueba</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>p4</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Revisión final (errores, coherencia, puntajes).</t>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -677,19 +677,19 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46150</v>
+        <v>46197</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>46148</v>
+        <v>46218</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>escanear</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -699,12 +699,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Escanear pruebas/controles y subir a carpeta.</t>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -715,34 +715,34 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46150</v>
+        <v>46202</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>46136</v>
+        <v>46216</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Trabajo práctico</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>revisar_tp</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sección 2</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>p6, p1</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Revisar TP y poner nota; subir rúbrica si aplica.</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -753,34 +753,34 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46162</v>
+        <v>46202</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>46148</v>
+        <v>46223</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>corregir_y_notas</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>p2</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Corrección por sección. Subir nota final.</t>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -791,10 +791,10 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46188</v>
+        <v>46202</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>46209</v>
+        <v>46216</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -803,22 +803,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>pedir_preguntas</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sección 1</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>p4, p5</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Preguntas para examen (temas por unidad).</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -829,10 +829,10 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46189</v>
+        <v>46202</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>46210</v>
+        <v>46223</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -856,7 +856,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Preguntas para examen (temas por unidad).</t>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -867,10 +867,10 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46190</v>
+        <v>46204</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>46211</v>
+        <v>46218</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -879,7 +879,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>pedir_preguntas</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -889,12 +889,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>p6, p1</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Preguntas para examen (temas por unidad).</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -905,10 +905,10 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46191</v>
+        <v>46204</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>46212</v>
+        <v>46225</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -922,7 +922,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Preguntas para examen (temas por unidad).</t>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -943,10 +943,10 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46195</v>
+        <v>46204</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>46209</v>
+        <v>46218</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -960,17 +960,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sección 1</t>
+          <t>Sección 4</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>p3, p1</t>
+          <t>p2, p4</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Construcción examen final + revisión cruzada.</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -981,10 +981,10 @@
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46196</v>
+        <v>46204</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>46210</v>
+        <v>46225</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -993,22 +993,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>construir_examen</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sección 2</t>
+          <t>Sección 4</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>p1, p2</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Construcción examen final + revisión cruzada.</t>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1019,10 +1019,10 @@
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46197</v>
+        <v>46209</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>46211</v>
+        <v>46216</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1031,22 +1031,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>construir_examen</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sección 3</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>p6, p5</t>
+          <t>p2, p5</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Construcción examen final + revisión cruzada.</t>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1057,10 +1057,10 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46198</v>
+        <v>46209</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>46212</v>
+        <v>46223</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1074,17 +1074,17 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>p4, p3</t>
+          <t>p3, p2</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Construcción examen final + revisión cruzada.</t>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1095,10 +1095,10 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46202</v>
+        <v>46209</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>46209</v>
+        <v>46216</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1112,17 +1112,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Sección 1</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>p6, p4</t>
+          <t>p1, p2</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pauta oficial examen.</t>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1133,10 +1133,10 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46203</v>
+        <v>46209</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>46210</v>
+        <v>46223</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>pauta_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1155,12 +1155,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>p3, p4</t>
+          <t>p4, p5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pauta oficial examen.</t>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1171,10 +1171,10 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46204</v>
+        <v>46211</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>46211</v>
+        <v>46218</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1193,12 +1193,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>p2, p6</t>
+          <t>p4, p3</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Pauta oficial examen.</t>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1209,10 +1209,10 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>46205</v>
+        <v>46211</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>46212</v>
+        <v>46225</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1221,22 +1221,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>pauta_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>p1, p3</t>
+          <t>p3, p6</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pauta oficial examen.</t>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1247,10 +1247,10 @@
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>46223</v>
+        <v>46211</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>46209</v>
+        <v>46218</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1259,22 +1259,22 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>corregir_examen</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sección 1</t>
+          <t>Sección 4</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>p1, p3</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Corrección examen por sección.</t>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1285,10 +1285,10 @@
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>46224</v>
+        <v>46211</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>46210</v>
+        <v>46225</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1297,22 +1297,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>corregir_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sección 2</t>
+          <t>Sección 4</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>p5, p3</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Corrección examen por sección.</t>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1323,10 +1323,10 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46225</v>
+        <v>46216</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>46211</v>
+        <v>46223</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1335,22 +1335,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>corregir_examen</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sección 3</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>p1</t>
+          <t>p3, p1</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Corrección examen por sección.</t>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1361,10 +1361,10 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46226</v>
+        <v>46216</v>
       </c>
       <c r="B24" s="3" t="n">
-        <v>46212</v>
+        <v>46223</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1373,32 +1373,412 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
+          <t>pauta_examen</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sección 2</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>p6, p5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>pauta_examen</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sección 3</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>p4, p5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>pauta_examen</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Sección 4</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>p4, p5</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
           <t>corregir_examen</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sección 1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>p4</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sección 2</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>46218</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sección 3</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>46218</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>Sección 4</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>p6</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Corrección examen por sección.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sección 1</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>p6</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sección 2</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>p2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sección 3</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>p2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Sección 4</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H24"/>
+  <autoFilter ref="A1:H34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1409,40 +1789,52 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="51" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Evaluaciones</t>
+          <t>Evaluación</t>
         </is>
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
-          <t>Sección 1 (lunes - DA)</t>
+          <t>Misión</t>
         </is>
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
-          <t>Sección 2 (viernes - JL)</t>
+          <t>Detalle</t>
         </is>
       </c>
       <c r="D1" s="4" t="inlineStr">
         <is>
-          <t>Sección 3 (martes - JL)</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Sección 4 (miércoles - ??)</t>
+          <t>Sección 2</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Sección 3</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Sección 4</t>
         </is>
       </c>
     </row>
@@ -1454,57 +1846,321 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>p1</t>
+          <t>p6, p1</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>p6</t>
+          <t>p4, p5</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>p6, p1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>p2, p4</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Prueba</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>construir_examen</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>p3, p2</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>p2</t>
+          <t>p4, p5</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>p3, p6</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>p5, p3</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>p4</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>p6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>p6</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>p2</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>p2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>pauta_examen</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>p2, p5</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>p1, p2</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>p4, p3</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>p1, p3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>pauta_examen</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>p3, p1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>p6, p5</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>p4, p5</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>p4, p5</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>pedir_preguntas</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>pedir_preguntas</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Todos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>Trabajo práctico</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>revisar_tp</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Revisar TP y poner nota. — Entrega al final</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E4"/>
+  <autoFilter ref="A1:G10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1515,16 +2171,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="51" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
@@ -1572,10 +2228,10 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="n">
-        <v>46188</v>
+        <v>46195</v>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46209</v>
+        <v>46216</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1599,7 +2255,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Preguntas para examen (temas por unidad).</t>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1610,10 +2266,10 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
-        <v>46189</v>
+        <v>46202</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>46210</v>
+        <v>46223</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -1627,7 +2283,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sección 2</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1637,7 +2293,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Preguntas para examen (temas por unidad).</t>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1648,10 +2304,10 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="n">
-        <v>46190</v>
+        <v>46195</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>46211</v>
+        <v>46216</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -1665,7 +2321,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Sección 3</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1675,7 +2331,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Preguntas para examen (temas por unidad).</t>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1686,10 +2342,10 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
-        <v>46191</v>
+        <v>46202</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>46212</v>
+        <v>46223</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -1703,7 +2359,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1713,7 +2369,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Preguntas para examen (temas por unidad).</t>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -1724,10 +2380,10 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
-        <v>46195</v>
+        <v>46197</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>46209</v>
+        <v>46218</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1736,22 +2392,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>construir_examen</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Sección 1</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>p3, p1</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Construcción examen final + revisión cruzada.</t>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1762,10 +2418,10 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
-        <v>46196</v>
+        <v>46204</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>46210</v>
+        <v>46225</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1774,22 +2430,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>construir_examen</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Sección 2</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>p1, p2</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Construcción examen final + revisión cruzada.</t>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1803,7 +2459,7 @@
         <v>46197</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>46211</v>
+        <v>46218</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1812,22 +2468,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>construir_examen</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Sección 3</t>
+          <t>Sección 4</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>p6, p5</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Construcción examen final + revisión cruzada.</t>
+          <t>Preguntas examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1838,10 +2494,10 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>46198</v>
+        <v>46204</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>46212</v>
+        <v>46225</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1850,7 +2506,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>construir_examen</t>
+          <t>pedir_preguntas</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1860,12 +2516,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>p4, p3</t>
+          <t>Todos</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Construcción examen final + revisión cruzada.</t>
+          <t>Preguntas examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1879,7 +2535,7 @@
         <v>46202</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>46209</v>
+        <v>46216</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1888,7 +2544,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>pauta_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1898,12 +2554,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>p6, p4</t>
+          <t>p6, p1</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Pauta oficial examen.</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1914,10 +2570,10 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>46203</v>
+        <v>46209</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>46210</v>
+        <v>46223</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1926,22 +2582,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>pauta_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Sección 2</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>p3, p4</t>
+          <t>p3, p2</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pauta oficial examen.</t>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1952,10 +2608,10 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>46204</v>
+        <v>46202</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>46211</v>
+        <v>46216</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1964,22 +2620,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>pauta_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sección 3</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>p2, p6</t>
+          <t>p4, p5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pauta oficial examen.</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1990,10 +2646,10 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>46205</v>
+        <v>46209</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>46212</v>
+        <v>46223</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -2002,22 +2658,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>pauta_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>p1, p3</t>
+          <t>p4, p5</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pauta oficial examen.</t>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -2028,10 +2684,10 @@
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>46223</v>
+        <v>46204</v>
       </c>
       <c r="B14" s="3" t="n">
-        <v>46209</v>
+        <v>46218</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -2040,22 +2696,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>corregir_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Sección 1</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>p6, p1</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Corrección examen por sección.</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -2066,10 +2722,10 @@
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>46224</v>
+        <v>46211</v>
       </c>
       <c r="B15" s="3" t="n">
-        <v>46210</v>
+        <v>46225</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -2078,22 +2734,22 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>corregir_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Sección 2</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>p5</t>
+          <t>p3, p6</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Corrección examen por sección.</t>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -2104,10 +2760,10 @@
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>46225</v>
+        <v>46204</v>
       </c>
       <c r="B16" s="3" t="n">
-        <v>46211</v>
+        <v>46218</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -2116,22 +2772,22 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>corregir_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sección 3</t>
+          <t>Sección 4</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>p1</t>
+          <t>p2, p4</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Corrección examen por sección.</t>
+          <t>Construcción examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -2142,10 +2798,10 @@
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>46226</v>
+        <v>46211</v>
       </c>
       <c r="B17" s="3" t="n">
-        <v>46212</v>
+        <v>46225</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2154,7 +2810,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>corregir_examen</t>
+          <t>construir_examen</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -2164,12 +2820,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>p6</t>
+          <t>p5, p3</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Corrección examen por sección.</t>
+          <t>Construcción examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -2180,34 +2836,34 @@
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>46134</v>
+        <v>46209</v>
       </c>
       <c r="B18" s="3" t="n">
-        <v>46148</v>
+        <v>46216</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>pedir_preguntas</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Todos</t>
+          <t>p2, p5</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Cada profesor: 2 alternativas + 1 desarrollo (según tema de la prueba).</t>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2218,34 +2874,34 @@
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>46141</v>
+        <v>46216</v>
       </c>
       <c r="B19" s="3" t="n">
-        <v>46148</v>
+        <v>46223</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>construir_control</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 1</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>p6, p1</t>
+          <t>p3, p1</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Armar versión final, diagramación y revisión cruzada.</t>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2256,34 +2912,34 @@
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>46143</v>
+        <v>46209</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>46148</v>
+        <v>46216</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>pauta_prueba</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>p2, p5</t>
+          <t>p1, p2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Pauta oficial: dividir en 2 mitades si son 2 responsables.</t>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2294,34 +2950,34 @@
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>46145</v>
+        <v>46216</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>46148</v>
+        <v>46223</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>revisar_prueba</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 2</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>p4</t>
+          <t>p6, p5</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Revisión final (errores, coherencia, puntajes).</t>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -2332,34 +2988,34 @@
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>46162</v>
+        <v>46211</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>46148</v>
+        <v>46218</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>corregir_y_notas</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>p2</t>
+          <t>p4, p3</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Corrección por sección. Subir nota final.</t>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2370,34 +3026,34 @@
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>46150</v>
+        <v>46218</v>
       </c>
       <c r="B23" s="3" t="n">
-        <v>46148</v>
+        <v>46225</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Prueba</t>
+          <t>Examen</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>escanear</t>
+          <t>pauta_examen</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Sección 4</t>
+          <t>Sección 3</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>p3</t>
+          <t>p4, p5</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Escanear pruebas/controles y subir a carpeta.</t>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2408,44 +3064,424 @@
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>46218</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>pauta_examen</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Sección 4</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>p1, p3</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pauta examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>pauta_examen</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Sección 4</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>p4, p5</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Pauta examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Sección 1</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>p4</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Sección 1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>p6</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>46230</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Sección 2</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>p3</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>46223</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Sección 2</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>p2</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>46218</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Sección 3</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Sección 3</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>p2</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>46232</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>46218</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Sección 4</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>p6</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Primera Oportunidad</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>46239</v>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>46225</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Examen</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>corregir_examen</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Sección 4</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>p1</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Corrección examen. — Examen Segunda Oportunidad</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
         <v>46150</v>
       </c>
-      <c r="B24" s="3" t="n">
+      <c r="B34" s="3" t="n">
         <v>46136</v>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>Trabajo práctico</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>revisar_tp</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Sección 2</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Revisar TP y poner nota; subir rúbrica si aplica.</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Revisar TP y poner nota. — Entrega al final</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H24"/>
+  <autoFilter ref="A1:H34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>